<commit_message>
Sprint 3 Day 17: Implement composite scoring and screener workbook export
</commit_message>
<xml_diff>
--- a/output/debt_free_blue_chip.xlsx
+++ b/output/debt_free_blue_chip.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V22"/>
+  <dimension ref="A1:Y22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,100 +429,115 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>cash_from_operations_cr</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>net_profit_margin_pct</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>return_on_equity_pct</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>debt_to_equity</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>interest_coverage</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>asset_turnover</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>free_cash_flow_cr</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>revenue_cagr_5yr</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>pat_cagr_5yr</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>eps_cagr_5yr</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>roce_percentage</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>market_cap_crore</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>pe_ratio</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>pb_ratio</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>dividend_yield_pct</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>net_profit</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>opm_percentage</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>broad_sector</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>dividend_payout_ratio_pct</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
         <is>
           <t>composite_quality_score</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>roce_percentage</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>market_cap_crore</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>pe_ratio</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>pb_ratio</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>dividend_yield_pct</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>net_profit</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>opm_percentage</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>broad_sector</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>dividend_payout_ratio_pct</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>sector_relative_score</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
         <is>
           <t>revenue_cagr_3yr</t>
         </is>
@@ -531,7 +546,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>LICI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -540,74 +555,81 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>27.85</v>
+        <v>26122</v>
       </c>
       <c r="D2" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="E2" t="n">
+        <v>49.45</v>
+      </c>
+      <c r="F2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>inf</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="G2" t="n">
-        <v>18742</v>
-      </c>
       <c r="H2" t="n">
-        <v>7.95</v>
+        <v>0.16</v>
       </c>
       <c r="I2" t="n">
-        <v>10.08</v>
+        <v>853</v>
       </c>
       <c r="J2" t="n">
-        <v>9.859999999999999</v>
+        <v>8.16</v>
       </c>
       <c r="K2" t="n">
-        <v>79.56</v>
-      </c>
-      <c r="L2" t="n">
-        <v>34.76</v>
-      </c>
+        <v>73.18000000000001</v>
+      </c>
+      <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
-        <v>332245.58</v>
+        <v>63.79</v>
       </c>
       <c r="N2" t="n">
-        <v>47.85</v>
+        <v>183583.67</v>
       </c>
       <c r="O2" t="n">
-        <v>3.24</v>
+        <v>30.67</v>
       </c>
       <c r="P2" t="n">
-        <v>4.26</v>
+        <v>8.1</v>
       </c>
       <c r="Q2" t="n">
-        <v>70866</v>
+        <v>3.77</v>
       </c>
       <c r="R2" t="n">
-        <v>20751</v>
+        <v>845966</v>
       </c>
       <c r="S2" t="n">
-        <v>37</v>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>Consumer Staples</t>
-        </is>
-      </c>
-      <c r="U2" t="n">
-        <v>84</v>
+        <v>40916</v>
+      </c>
+      <c r="T2" t="n">
+        <v>4</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
       </c>
       <c r="V2" t="n">
-        <v>12.89030700491063</v>
+        <v>15</v>
+      </c>
+      <c r="W2" t="n">
+        <v>69.35193867952822</v>
+      </c>
+      <c r="X2" t="n">
+        <v>100</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>6.981735429882496</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ICICIGI</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -616,74 +638,83 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>15.72</v>
+        <v>17179</v>
       </c>
       <c r="D3" t="n">
+        <v>29.28</v>
+      </c>
+      <c r="E3" t="n">
+        <v>27.85</v>
+      </c>
+      <c r="F3" t="n">
         <v>0</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>inf</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="G3" t="n">
-        <v>486</v>
-      </c>
       <c r="H3" t="n">
-        <v>12.91</v>
+        <v>0.77</v>
       </c>
       <c r="I3" t="n">
-        <v>12.84</v>
+        <v>18742</v>
       </c>
       <c r="J3" t="n">
-        <v>11.14</v>
+        <v>7.95</v>
       </c>
       <c r="K3" t="n">
-        <v>72.98</v>
+        <v>10.08</v>
       </c>
       <c r="L3" t="n">
-        <v>22.5</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="M3" t="n">
-        <v>1271789.21</v>
+        <v>34.76</v>
       </c>
       <c r="N3" t="n">
-        <v>49</v>
+        <v>332245.58</v>
       </c>
       <c r="O3" t="n">
-        <v>7.86</v>
+        <v>47.85</v>
       </c>
       <c r="P3" t="n">
-        <v>3.46</v>
+        <v>3.24</v>
       </c>
       <c r="Q3" t="n">
-        <v>20487</v>
+        <v>4.26</v>
       </c>
       <c r="R3" t="n">
-        <v>1919</v>
+        <v>70866</v>
       </c>
       <c r="S3" t="n">
-        <v>2577</v>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="U3" t="n">
-        <v>28</v>
+        <v>20751</v>
+      </c>
+      <c r="T3" t="n">
+        <v>37</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
       </c>
       <c r="V3" t="n">
-        <v>18.98796206427069</v>
+        <v>84</v>
+      </c>
+      <c r="W3" t="n">
+        <v>62.56179668427612</v>
+      </c>
+      <c r="X3" t="n">
+        <v>86.1627693924593</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>12.89030700491063</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LICI</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -692,72 +723,81 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>49.45</v>
+        <v>-72760</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+        <v>26.29</v>
+      </c>
+      <c r="E4" t="n">
+        <v>18.84</v>
       </c>
       <c r="F4" t="n">
-        <v>0.16</v>
+        <v>3.82</v>
       </c>
       <c r="G4" t="n">
-        <v>853</v>
+        <v>2689.17</v>
       </c>
       <c r="H4" t="n">
-        <v>8.16</v>
+        <v>0.15</v>
       </c>
       <c r="I4" t="n">
-        <v>73.18000000000001</v>
-      </c>
-      <c r="J4" t="inlineStr"/>
+        <v>-79931</v>
+      </c>
+      <c r="J4" t="n">
+        <v>24.35</v>
+      </c>
       <c r="K4" t="n">
-        <v>69.53</v>
+        <v>29.32</v>
       </c>
       <c r="L4" t="n">
-        <v>63.79</v>
+        <v>27.56</v>
       </c>
       <c r="M4" t="n">
-        <v>183583.67</v>
+        <v>11.9</v>
       </c>
       <c r="N4" t="n">
-        <v>30.67</v>
+        <v>2473271.58</v>
       </c>
       <c r="O4" t="n">
-        <v>8.1</v>
+        <v>69.2</v>
       </c>
       <c r="P4" t="n">
-        <v>3.77</v>
+        <v>4.11</v>
       </c>
       <c r="Q4" t="n">
-        <v>845966</v>
+        <v>0.27</v>
       </c>
       <c r="R4" t="n">
-        <v>40916</v>
+        <v>54972</v>
       </c>
       <c r="S4" t="n">
-        <v>4</v>
-      </c>
-      <c r="T4" t="inlineStr">
+        <v>14451</v>
+      </c>
+      <c r="T4" t="n">
+        <v>19987</v>
+      </c>
+      <c r="U4" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="U4" t="n">
+      <c r="V4" t="n">
         <v>15</v>
       </c>
-      <c r="V4" t="n">
-        <v>6.981735429882496</v>
+      <c r="W4" t="n">
+        <v>53.93087060072213</v>
+      </c>
+      <c r="X4" t="n">
+        <v>56.74930782316123</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>27.25940575809531</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>ICICIGI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -766,74 +806,83 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>20.64</v>
+        <v>2407</v>
       </c>
       <c r="D5" t="n">
+        <v>9.369999999999999</v>
+      </c>
+      <c r="E5" t="n">
+        <v>15.72</v>
+      </c>
+      <c r="F5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>inf</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1536</v>
-      </c>
       <c r="H5" t="n">
-        <v>6.72</v>
+        <v>0.32</v>
       </c>
       <c r="I5" t="n">
-        <v>9.279999999999999</v>
+        <v>486</v>
       </c>
       <c r="J5" t="n">
-        <v>9.26</v>
+        <v>12.91</v>
       </c>
       <c r="K5" t="n">
-        <v>68.12</v>
+        <v>12.84</v>
       </c>
       <c r="L5" t="n">
-        <v>20.6</v>
+        <v>11.14</v>
       </c>
       <c r="M5" t="n">
-        <v>2599556.05</v>
+        <v>22.5</v>
       </c>
       <c r="N5" t="n">
-        <v>58.43</v>
+        <v>1271789.21</v>
       </c>
       <c r="O5" t="n">
-        <v>6.47</v>
+        <v>49</v>
       </c>
       <c r="P5" t="n">
-        <v>4.23</v>
+        <v>7.86</v>
       </c>
       <c r="Q5" t="n">
-        <v>16727</v>
+        <v>3.46</v>
       </c>
       <c r="R5" t="n">
-        <v>2490</v>
+        <v>20487</v>
       </c>
       <c r="S5" t="n">
-        <v>13</v>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
-      <c r="U5" t="n">
-        <v>44</v>
+        <v>1919</v>
+      </c>
+      <c r="T5" t="n">
+        <v>2577</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
       </c>
       <c r="V5" t="n">
-        <v>19.843289373664</v>
+        <v>28</v>
+      </c>
+      <c r="W5" t="n">
+        <v>49.39652873350715</v>
+      </c>
+      <c r="X5" t="n">
+        <v>44.03206779015759</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>18.98796206427069</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -842,74 +891,81 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>15.75</v>
+        <v>157284</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+        <v>28.89</v>
+      </c>
+      <c r="E6" t="n">
+        <v>17.99</v>
       </c>
       <c r="F6" t="n">
-        <v>1.23</v>
+        <v>6.45</v>
       </c>
       <c r="G6" t="n">
-        <v>4936</v>
+        <v>1.3</v>
       </c>
       <c r="H6" t="n">
-        <v>10.51</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I6" t="n">
-        <v>12.01</v>
+        <v>12547</v>
       </c>
       <c r="J6" t="n">
-        <v>11.14</v>
+        <v>17.25</v>
       </c>
       <c r="K6" t="n">
-        <v>67.33</v>
+        <v>51.95</v>
       </c>
       <c r="L6" t="n">
-        <v>23.67</v>
+        <v>55.18</v>
       </c>
       <c r="M6" t="n">
-        <v>1503863.63</v>
+        <v>7.6</v>
       </c>
       <c r="N6" t="n">
-        <v>20.78</v>
+        <v>1319221.86</v>
       </c>
       <c r="O6" t="n">
-        <v>8.26</v>
+        <v>25.76</v>
       </c>
       <c r="P6" t="n">
-        <v>1.78</v>
+        <v>6.2</v>
       </c>
       <c r="Q6" t="n">
-        <v>141858</v>
+        <v>3.43</v>
       </c>
       <c r="R6" t="n">
-        <v>13488</v>
+        <v>159516</v>
       </c>
       <c r="S6" t="n">
-        <v>13</v>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
-      <c r="U6" t="n">
-        <v>29</v>
+        <v>46081</v>
+      </c>
+      <c r="T6" t="n">
+        <v>-14152</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
       </c>
       <c r="V6" t="n">
-        <v>26.32364432616601</v>
+        <v>16</v>
+      </c>
+      <c r="W6" t="n">
+        <v>48.83992353907501</v>
+      </c>
+      <c r="X6" t="n">
+        <v>42.47098526296872</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>21.39660074377121</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -918,72 +974,83 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>14.01</v>
+        <v>16801</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>9.51</v>
       </c>
       <c r="E7" t="n">
-        <v>1.24</v>
+        <v>15.75</v>
       </c>
       <c r="F7" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="G7" t="n">
-        <v>6766</v>
+        <v>0</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="H7" t="n">
-        <v>13.52</v>
+        <v>1.23</v>
       </c>
       <c r="I7" t="n">
-        <v>20.38</v>
+        <v>4936</v>
       </c>
       <c r="J7" t="n">
-        <v>19.34</v>
+        <v>10.51</v>
       </c>
       <c r="K7" t="n">
-        <v>65.58</v>
+        <v>12.01</v>
       </c>
       <c r="L7" t="n">
-        <v>7.86</v>
+        <v>11.14</v>
       </c>
       <c r="M7" t="n">
-        <v>430223.52</v>
+        <v>23.67</v>
       </c>
       <c r="N7" t="n">
-        <v>32.9</v>
+        <v>1503863.63</v>
       </c>
       <c r="O7" t="n">
-        <v>1.15</v>
+        <v>20.78</v>
       </c>
       <c r="P7" t="n">
-        <v>1.51</v>
+        <v>8.26</v>
       </c>
       <c r="Q7" t="n">
-        <v>56237</v>
+        <v>1.78</v>
       </c>
       <c r="R7" t="n">
-        <v>18213</v>
+        <v>141858</v>
       </c>
       <c r="S7" t="n">
-        <v>-13382</v>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="U7" t="n">
-        <v>2</v>
+        <v>13488</v>
+      </c>
+      <c r="T7" t="n">
+        <v>13</v>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
       </c>
       <c r="V7" t="n">
-        <v>19.66335897034557</v>
+        <v>29</v>
+      </c>
+      <c r="W7" t="n">
+        <v>46.94201315314325</v>
+      </c>
+      <c r="X7" t="n">
+        <v>31.86080183638076</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>26.32364432616601</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -992,66 +1059,81 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>61.32</v>
+        <v>-68674</v>
       </c>
       <c r="D8" t="n">
-        <v>3.68</v>
+        <v>14.13</v>
       </c>
       <c r="E8" t="n">
+        <v>25.85</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="H8" t="n">
         <v>0.21</v>
       </c>
-      <c r="F8" t="n">
-        <v>1.51</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-29445</v>
-      </c>
-      <c r="H8" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
+      <c r="I8" t="n">
+        <v>-79634</v>
+      </c>
+      <c r="J8" t="n">
+        <v>20.97</v>
+      </c>
       <c r="K8" t="n">
-        <v>64.92</v>
+        <v>23.75</v>
       </c>
       <c r="L8" t="n">
-        <v>1.63</v>
+        <v>20.59</v>
       </c>
       <c r="M8" t="n">
-        <v>1825925.6</v>
+        <v>21.14</v>
       </c>
       <c r="N8" t="n">
-        <v>19.29</v>
+        <v>1905112.17</v>
       </c>
       <c r="O8" t="n">
-        <v>10.91</v>
+        <v>15.07</v>
       </c>
       <c r="P8" t="n">
-        <v>1.32</v>
+        <v>6.08</v>
       </c>
       <c r="Q8" t="n">
-        <v>109065</v>
+        <v>2.56</v>
       </c>
       <c r="R8" t="n">
-        <v>9157</v>
-      </c>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr">
+        <v>110382</v>
+      </c>
+      <c r="S8" t="n">
+        <v>15595</v>
+      </c>
+      <c r="T8" t="n">
+        <v>37</v>
+      </c>
+      <c r="U8" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="U8" t="n">
-        <v>18</v>
-      </c>
       <c r="V8" t="n">
-        <v>10.00319904301221</v>
+        <v>2</v>
+      </c>
+      <c r="W8" t="n">
+        <v>46.36161820089244</v>
+      </c>
+      <c r="X8" t="n">
+        <v>35.52020722644187</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>22.13149041552844</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1060,72 +1142,83 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>17.99</v>
+        <v>1253</v>
       </c>
       <c r="D9" t="n">
-        <v>6.45</v>
+        <v>14.89</v>
       </c>
       <c r="E9" t="n">
-        <v>1.3</v>
+        <v>20.64</v>
       </c>
       <c r="F9" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="G9" t="n">
-        <v>12547</v>
+        <v>0</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="H9" t="n">
-        <v>17.25</v>
+        <v>0.96</v>
       </c>
       <c r="I9" t="n">
-        <v>51.95</v>
+        <v>1536</v>
       </c>
       <c r="J9" t="n">
-        <v>55.18</v>
+        <v>6.72</v>
       </c>
       <c r="K9" t="n">
-        <v>63.6</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="L9" t="n">
-        <v>7.6</v>
+        <v>9.26</v>
       </c>
       <c r="M9" t="n">
-        <v>1319221.86</v>
+        <v>20.6</v>
       </c>
       <c r="N9" t="n">
-        <v>25.76</v>
+        <v>2599556.05</v>
       </c>
       <c r="O9" t="n">
-        <v>6.2</v>
+        <v>58.43</v>
       </c>
       <c r="P9" t="n">
-        <v>3.43</v>
+        <v>6.47</v>
       </c>
       <c r="Q9" t="n">
-        <v>159516</v>
+        <v>4.23</v>
       </c>
       <c r="R9" t="n">
-        <v>46081</v>
+        <v>16727</v>
       </c>
       <c r="S9" t="n">
-        <v>-14152</v>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="U9" t="n">
-        <v>16</v>
+        <v>2490</v>
+      </c>
+      <c r="T9" t="n">
+        <v>13</v>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
       </c>
       <c r="V9" t="n">
-        <v>21.39660074377121</v>
+        <v>44</v>
+      </c>
+      <c r="W9" t="n">
+        <v>45.64309856903565</v>
+      </c>
+      <c r="X9" t="n">
+        <v>28.60157906204023</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>19.843289373664</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1134,72 +1227,81 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>15.83</v>
+        <v>15685</v>
       </c>
       <c r="D10" t="n">
-        <v>8.25</v>
+        <v>32.39</v>
       </c>
       <c r="E10" t="n">
-        <v>1.69</v>
+        <v>14.01</v>
       </c>
       <c r="F10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="H10" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="G10" t="n">
-        <v>-14556</v>
-      </c>
-      <c r="H10" t="n">
-        <v>14.74</v>
-      </c>
       <c r="I10" t="n">
-        <v>39.67</v>
+        <v>6766</v>
       </c>
       <c r="J10" t="n">
-        <v>35.1</v>
+        <v>13.52</v>
       </c>
       <c r="K10" t="n">
-        <v>60.76</v>
+        <v>20.38</v>
       </c>
       <c r="L10" t="n">
-        <v>7.06</v>
+        <v>19.34</v>
       </c>
       <c r="M10" t="n">
-        <v>948868.63</v>
+        <v>7.86</v>
       </c>
       <c r="N10" t="n">
-        <v>38.14</v>
+        <v>430223.52</v>
       </c>
       <c r="O10" t="n">
-        <v>4.66</v>
+        <v>32.9</v>
       </c>
       <c r="P10" t="n">
-        <v>2.32</v>
+        <v>1.15</v>
       </c>
       <c r="Q10" t="n">
-        <v>109369</v>
+        <v>1.51</v>
       </c>
       <c r="R10" t="n">
-        <v>24861</v>
+        <v>56237</v>
       </c>
       <c r="S10" t="n">
-        <v>11952</v>
-      </c>
-      <c r="T10" t="inlineStr">
+        <v>18213</v>
+      </c>
+      <c r="T10" t="n">
+        <v>-13382</v>
+      </c>
+      <c r="U10" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="U10" t="n">
-        <v>1</v>
-      </c>
       <c r="V10" t="n">
-        <v>19.96604689042871</v>
+        <v>2</v>
+      </c>
+      <c r="W10" t="n">
+        <v>44.60816379359672</v>
+      </c>
+      <c r="X10" t="n">
+        <v>30.60238205191349</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>19.66335897034557</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CANBK</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1208,72 +1310,81 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>16.72</v>
+        <v>19069</v>
       </c>
       <c r="D11" t="n">
-        <v>14.87</v>
+        <v>23.07</v>
       </c>
       <c r="E11" t="n">
-        <v>1.61</v>
+        <v>14.34</v>
       </c>
       <c r="F11" t="n">
+        <v>6.81</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H11" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="G11" t="n">
-        <v>13296</v>
-      </c>
-      <c r="H11" t="n">
-        <v>18.18</v>
-      </c>
       <c r="I11" t="n">
-        <v>85.78</v>
+        <v>35669</v>
       </c>
       <c r="J11" t="n">
-        <v>53.42</v>
+        <v>21.95</v>
       </c>
       <c r="K11" t="n">
-        <v>59.34</v>
+        <v>23.87</v>
       </c>
       <c r="L11" t="n">
-        <v>6.63</v>
+        <v>15.42</v>
       </c>
       <c r="M11" t="n">
-        <v>496415.88</v>
+        <v>7.67</v>
       </c>
       <c r="N11" t="n">
-        <v>36.74</v>
+        <v>808359.03</v>
       </c>
       <c r="O11" t="n">
-        <v>12.61</v>
+        <v>49.42</v>
       </c>
       <c r="P11" t="n">
-        <v>3.81</v>
+        <v>4.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>110519</v>
+        <v>4.33</v>
       </c>
       <c r="R11" t="n">
-        <v>15401</v>
+        <v>283649</v>
       </c>
       <c r="S11" t="n">
-        <v>-7745</v>
-      </c>
-      <c r="T11" t="inlineStr">
+        <v>65446</v>
+      </c>
+      <c r="T11" t="n">
+        <v>-44685</v>
+      </c>
+      <c r="U11" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="U11" t="n">
-        <v>19</v>
-      </c>
       <c r="V11" t="n">
-        <v>16.30293930023252</v>
+        <v>23</v>
+      </c>
+      <c r="W11" t="n">
+        <v>44.08554497818926</v>
+      </c>
+      <c r="X11" t="n">
+        <v>29.13661940852842</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>30.18695614094877</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1282,72 +1393,83 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>18.84</v>
+        <v>29122</v>
       </c>
       <c r="D12" t="n">
-        <v>3.82</v>
+        <v>1.43</v>
       </c>
       <c r="E12" t="n">
-        <v>2689.17</v>
+        <v>12.7</v>
       </c>
       <c r="F12" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="G12" t="n">
-        <v>-79931</v>
+        <v>0</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="H12" t="n">
-        <v>24.35</v>
+        <v>0.33</v>
       </c>
       <c r="I12" t="n">
-        <v>29.32</v>
+        <v>-2099</v>
       </c>
       <c r="J12" t="n">
-        <v>27.56</v>
+        <v>24.23</v>
       </c>
       <c r="K12" t="n">
-        <v>57.47</v>
+        <v>7.37</v>
       </c>
       <c r="L12" t="n">
-        <v>11.9</v>
+        <v>7.89</v>
       </c>
       <c r="M12" t="n">
-        <v>2473271.58</v>
+        <v>13.2</v>
       </c>
       <c r="N12" t="n">
-        <v>69.2</v>
+        <v>886097.71</v>
       </c>
       <c r="O12" t="n">
-        <v>4.11</v>
+        <v>69.98</v>
       </c>
       <c r="P12" t="n">
-        <v>0.27</v>
+        <v>9.48</v>
       </c>
       <c r="Q12" t="n">
-        <v>54972</v>
+        <v>1.62</v>
       </c>
       <c r="R12" t="n">
-        <v>14451</v>
+        <v>131988</v>
       </c>
       <c r="S12" t="n">
-        <v>19987</v>
-      </c>
-      <c r="T12" t="inlineStr">
+        <v>1894</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="U12" t="n">
-        <v>15</v>
-      </c>
       <c r="V12" t="n">
-        <v>27.25940575809531</v>
+        <v>14</v>
+      </c>
+      <c r="W12" t="n">
+        <v>43.11204743944869</v>
+      </c>
+      <c r="X12" t="n">
+        <v>26.40629994117292</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>17.23587757712</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>CANBK</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1356,72 +1478,81 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>25.85</v>
+        <v>15046</v>
       </c>
       <c r="D13" t="n">
-        <v>4.79</v>
+        <v>13.94</v>
       </c>
       <c r="E13" t="n">
-        <v>2.2</v>
+        <v>16.72</v>
       </c>
       <c r="F13" t="n">
-        <v>0.21</v>
+        <v>14.87</v>
       </c>
       <c r="G13" t="n">
-        <v>-79634</v>
+        <v>1.61</v>
       </c>
       <c r="H13" t="n">
-        <v>20.97</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I13" t="n">
-        <v>23.75</v>
+        <v>13296</v>
       </c>
       <c r="J13" t="n">
-        <v>20.59</v>
+        <v>18.18</v>
       </c>
       <c r="K13" t="n">
-        <v>56.77</v>
+        <v>85.78</v>
       </c>
       <c r="L13" t="n">
-        <v>21.14</v>
+        <v>53.42</v>
       </c>
       <c r="M13" t="n">
-        <v>1905112.17</v>
+        <v>6.63</v>
       </c>
       <c r="N13" t="n">
-        <v>15.07</v>
+        <v>496415.88</v>
       </c>
       <c r="O13" t="n">
-        <v>6.08</v>
+        <v>36.74</v>
       </c>
       <c r="P13" t="n">
-        <v>2.56</v>
+        <v>12.61</v>
       </c>
       <c r="Q13" t="n">
-        <v>110382</v>
+        <v>3.81</v>
       </c>
       <c r="R13" t="n">
-        <v>15595</v>
+        <v>110519</v>
       </c>
       <c r="S13" t="n">
-        <v>37</v>
-      </c>
-      <c r="T13" t="inlineStr">
+        <v>15401</v>
+      </c>
+      <c r="T13" t="n">
+        <v>-7745</v>
+      </c>
+      <c r="U13" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="U13" t="n">
-        <v>2</v>
-      </c>
       <c r="V13" t="n">
-        <v>22.13149041552844</v>
+        <v>19</v>
+      </c>
+      <c r="W13" t="n">
+        <v>42.60305121511472</v>
+      </c>
+      <c r="X13" t="n">
+        <v>24.97874389217935</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>16.30293930023252</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>IRFC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1430,68 +1561,75 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>12.7</v>
+        <v>7914</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+        <v>24.06</v>
+      </c>
+      <c r="E14" t="n">
+        <v>13.04</v>
       </c>
       <c r="F14" t="n">
-        <v>0.33</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>-2099</v>
+        <v>1.32</v>
       </c>
       <c r="H14" t="n">
-        <v>24.23</v>
+        <v>0.05</v>
       </c>
       <c r="I14" t="n">
-        <v>7.37</v>
+        <v>7906</v>
       </c>
       <c r="J14" t="n">
-        <v>7.89</v>
+        <v>19.07</v>
       </c>
       <c r="K14" t="n">
-        <v>55.2</v>
+        <v>23.25</v>
       </c>
       <c r="L14" t="n">
-        <v>13.2</v>
+        <v>20.11</v>
       </c>
       <c r="M14" t="n">
-        <v>886097.71</v>
+        <v>5.73</v>
       </c>
       <c r="N14" t="n">
-        <v>69.98</v>
+        <v>2618348.58</v>
       </c>
       <c r="O14" t="n">
-        <v>9.48</v>
+        <v>9.81</v>
       </c>
       <c r="P14" t="n">
-        <v>1.62</v>
+        <v>3.91</v>
       </c>
       <c r="Q14" t="n">
-        <v>131988</v>
+        <v>2.82</v>
       </c>
       <c r="R14" t="n">
-        <v>1894</v>
+        <v>26645</v>
       </c>
       <c r="S14" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" t="inlineStr">
+        <v>6412</v>
+      </c>
+      <c r="T14" t="n">
+        <v>100</v>
+      </c>
+      <c r="U14" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="U14" t="n">
-        <v>14</v>
-      </c>
       <c r="V14" t="n">
-        <v>17.23587757712</v>
+        <v>31</v>
+      </c>
+      <c r="W14" t="n">
+        <v>42.28401740380991</v>
+      </c>
+      <c r="X14" t="n">
+        <v>24.08396584592249</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>19.10193873049559</v>
       </c>
     </row>
     <row r="15">
@@ -1506,72 +1644,81 @@
         </is>
       </c>
       <c r="C15" t="n">
+        <v>-31101</v>
+      </c>
+      <c r="D15" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="E15" t="n">
         <v>15.12</v>
       </c>
-      <c r="D15" t="n">
+      <c r="F15" t="n">
         <v>3.99</v>
       </c>
-      <c r="E15" t="n">
+      <c r="G15" t="n">
         <v>0.68</v>
       </c>
-      <c r="F15" t="n">
+      <c r="H15" t="n">
         <v>0.15</v>
       </c>
-      <c r="G15" t="n">
+      <c r="I15" t="n">
         <v>-31359</v>
       </c>
-      <c r="H15" t="n">
+      <c r="J15" t="n">
         <v>18.56</v>
       </c>
-      <c r="I15" t="n">
+      <c r="K15" t="n">
         <v>23.49</v>
       </c>
-      <c r="J15" t="n">
+      <c r="L15" t="n">
         <v>14.29</v>
       </c>
-      <c r="K15" t="n">
-        <v>53.19</v>
-      </c>
-      <c r="L15" t="n">
+      <c r="M15" t="n">
         <v>11.3</v>
       </c>
-      <c r="M15" t="n">
+      <c r="N15" t="n">
         <v>868933.47</v>
       </c>
-      <c r="N15" t="n">
+      <c r="O15" t="n">
         <v>68.53</v>
       </c>
-      <c r="O15" t="n">
+      <c r="P15" t="n">
         <v>7.91</v>
       </c>
-      <c r="P15" t="n">
+      <c r="Q15" t="n">
         <v>1.86</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="R15" t="n">
         <v>36388</v>
       </c>
-      <c r="R15" t="n">
+      <c r="S15" t="n">
         <v>7399</v>
       </c>
-      <c r="S15" t="n">
+      <c r="T15" t="n">
         <v>29</v>
       </c>
-      <c r="T15" t="inlineStr">
+      <c r="U15" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="U15" t="n">
+      <c r="V15" t="n">
         <v>23</v>
       </c>
-      <c r="V15" t="n">
+      <c r="W15" t="n">
+        <v>41.51941759234256</v>
+      </c>
+      <c r="X15" t="n">
+        <v>21.93953130252711</v>
+      </c>
+      <c r="Y15" t="n">
         <v>27.82625310142639</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>PNB</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1580,72 +1727,75 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>14.25</v>
+        <v>-27939</v>
       </c>
       <c r="D16" t="n">
-        <v>6.89</v>
+        <v>8.4</v>
       </c>
       <c r="E16" t="n">
-        <v>1.88</v>
+        <v>61.32</v>
       </c>
       <c r="F16" t="n">
-        <v>0.09</v>
+        <v>3.68</v>
       </c>
       <c r="G16" t="n">
-        <v>-17468</v>
+        <v>0.21</v>
       </c>
       <c r="H16" t="n">
-        <v>15.5</v>
+        <v>1.51</v>
       </c>
       <c r="I16" t="n">
-        <v>22.08</v>
+        <v>-29445</v>
       </c>
       <c r="J16" t="n">
         <v>15.9</v>
       </c>
-      <c r="K16" t="n">
-        <v>52.45</v>
-      </c>
-      <c r="L16" t="n">
-        <v>7.93</v>
-      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
-        <v>1807433.12</v>
+        <v>1.63</v>
       </c>
       <c r="N16" t="n">
-        <v>8.99</v>
+        <v>1825925.6</v>
       </c>
       <c r="O16" t="n">
-        <v>3.7</v>
+        <v>19.29</v>
       </c>
       <c r="P16" t="n">
-        <v>1.42</v>
+        <v>10.91</v>
       </c>
       <c r="Q16" t="n">
-        <v>45748</v>
+        <v>1.32</v>
       </c>
       <c r="R16" t="n">
-        <v>8950</v>
+        <v>109065</v>
       </c>
       <c r="S16" t="n">
-        <v>2978</v>
-      </c>
-      <c r="T16" t="inlineStr">
+        <v>9157</v>
+      </c>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="U16" t="n">
-        <v>14</v>
-      </c>
       <c r="V16" t="n">
-        <v>16.41029009859514</v>
+        <v>18</v>
+      </c>
+      <c r="W16" t="n">
+        <v>40.07886946297909</v>
+      </c>
+      <c r="X16" t="n">
+        <v>17.89929859032939</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>10.00319904301221</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IRFC</t>
+          <t>CHOLAFIN</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1654,72 +1804,81 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>13.04</v>
+        <v>-35683</v>
       </c>
       <c r="D17" t="n">
-        <v>8.380000000000001</v>
+        <v>17.85</v>
       </c>
       <c r="E17" t="n">
-        <v>1.32</v>
+        <v>17.46</v>
       </c>
       <c r="F17" t="n">
-        <v>0.05</v>
+        <v>6.86</v>
       </c>
       <c r="G17" t="n">
-        <v>7906</v>
+        <v>21.21</v>
       </c>
       <c r="H17" t="n">
-        <v>19.07</v>
+        <v>0.12</v>
       </c>
       <c r="I17" t="n">
-        <v>23.25</v>
+        <v>-38538</v>
       </c>
       <c r="J17" t="n">
-        <v>20.11</v>
+        <v>21.94</v>
       </c>
       <c r="K17" t="n">
-        <v>49.7</v>
+        <v>23.36</v>
       </c>
       <c r="L17" t="n">
-        <v>5.73</v>
+        <v>22.28</v>
       </c>
       <c r="M17" t="n">
-        <v>2618348.58</v>
+        <v>10.4</v>
       </c>
       <c r="N17" t="n">
-        <v>9.81</v>
+        <v>971931.96</v>
       </c>
       <c r="O17" t="n">
-        <v>3.91</v>
+        <v>16.79</v>
       </c>
       <c r="P17" t="n">
-        <v>2.82</v>
+        <v>10.36</v>
       </c>
       <c r="Q17" t="n">
-        <v>26645</v>
+        <v>2.83</v>
       </c>
       <c r="R17" t="n">
-        <v>6412</v>
+        <v>19163</v>
       </c>
       <c r="S17" t="n">
-        <v>100</v>
-      </c>
-      <c r="T17" t="inlineStr">
+        <v>3420</v>
+      </c>
+      <c r="T17" t="n">
+        <v>4548</v>
+      </c>
+      <c r="U17" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="U17" t="n">
-        <v>31</v>
-      </c>
       <c r="V17" t="n">
-        <v>19.10193873049559</v>
+        <v>5</v>
+      </c>
+      <c r="W17" t="n">
+        <v>39.32907228731637</v>
+      </c>
+      <c r="X17" t="n">
+        <v>15.79638025329019</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>25.98553091668698</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PFC</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1728,72 +1887,81 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>26.16</v>
+        <v>-5555</v>
       </c>
       <c r="D18" t="n">
-        <v>8.52</v>
+        <v>22.73</v>
       </c>
       <c r="E18" t="n">
-        <v>0.58</v>
+        <v>15.83</v>
       </c>
       <c r="F18" t="n">
-        <v>0.09</v>
+        <v>8.25</v>
       </c>
       <c r="G18" t="n">
-        <v>-101229</v>
+        <v>1.69</v>
       </c>
       <c r="H18" t="n">
-        <v>11.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I18" t="n">
-        <v>15.92</v>
+        <v>-14556</v>
       </c>
       <c r="J18" t="n">
-        <v>14.87</v>
+        <v>14.74</v>
       </c>
       <c r="K18" t="n">
-        <v>49.31</v>
+        <v>39.67</v>
       </c>
       <c r="L18" t="n">
-        <v>9.960000000000001</v>
+        <v>35.1</v>
       </c>
       <c r="M18" t="n">
-        <v>2011885.81</v>
+        <v>7.06</v>
       </c>
       <c r="N18" t="n">
-        <v>35.6</v>
+        <v>948868.63</v>
       </c>
       <c r="O18" t="n">
-        <v>6.59</v>
+        <v>38.14</v>
       </c>
       <c r="P18" t="n">
-        <v>0.42</v>
+        <v>4.66</v>
       </c>
       <c r="Q18" t="n">
-        <v>91508</v>
+        <v>2.32</v>
       </c>
       <c r="R18" t="n">
-        <v>26461</v>
+        <v>109369</v>
       </c>
       <c r="S18" t="n">
-        <v>37</v>
-      </c>
-      <c r="T18" t="inlineStr">
+        <v>24861</v>
+      </c>
+      <c r="T18" t="n">
+        <v>11952</v>
+      </c>
+      <c r="U18" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="U18" t="n">
-        <v>23</v>
-      </c>
       <c r="V18" t="n">
-        <v>8.493112204756725</v>
+        <v>1</v>
+      </c>
+      <c r="W18" t="n">
+        <v>38.74446194015888</v>
+      </c>
+      <c r="X18" t="n">
+        <v>14.15675308615164</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>19.96604689042871</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BANKBARODA</t>
+          <t>RECLTD</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1802,72 +1970,81 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>15.76</v>
+        <v>-57723</v>
       </c>
       <c r="D19" t="n">
-        <v>12.14</v>
+        <v>29.77</v>
       </c>
       <c r="E19" t="n">
-        <v>1.9</v>
+        <v>20.4</v>
       </c>
       <c r="F19" t="n">
-        <v>0.07000000000000001</v>
+        <v>6.42</v>
       </c>
       <c r="G19" t="n">
-        <v>-7559</v>
+        <v>1.6</v>
       </c>
       <c r="H19" t="n">
-        <v>17.48</v>
+        <v>0.09</v>
       </c>
       <c r="I19" t="n">
-        <v>74.51000000000001</v>
+        <v>-59554</v>
       </c>
       <c r="J19" t="n">
-        <v>55.18</v>
+        <v>13.34</v>
       </c>
       <c r="K19" t="n">
-        <v>49.07</v>
+        <v>19.76</v>
       </c>
       <c r="L19" t="n">
-        <v>6.33</v>
+        <v>19.67</v>
       </c>
       <c r="M19" t="n">
-        <v>590971.02</v>
+        <v>10</v>
       </c>
       <c r="N19" t="n">
-        <v>16.89</v>
+        <v>291917.42</v>
       </c>
       <c r="O19" t="n">
-        <v>4.15</v>
+        <v>31.49</v>
       </c>
       <c r="P19" t="n">
-        <v>2.62</v>
+        <v>4.59</v>
       </c>
       <c r="Q19" t="n">
-        <v>118379</v>
+        <v>2.18</v>
       </c>
       <c r="R19" t="n">
-        <v>18869</v>
+        <v>47517</v>
       </c>
       <c r="S19" t="n">
-        <v>4102</v>
-      </c>
-      <c r="T19" t="inlineStr">
+        <v>14145</v>
+      </c>
+      <c r="T19" t="n">
+        <v>101</v>
+      </c>
+      <c r="U19" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="U19" t="n">
-        <v>21</v>
-      </c>
       <c r="V19" t="n">
-        <v>16.78883948962531</v>
+        <v>30</v>
+      </c>
+      <c r="W19" t="n">
+        <v>38.60551022458641</v>
+      </c>
+      <c r="X19" t="n">
+        <v>13.76704221483216</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>10.14749732259019</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>PFC</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1876,72 +2053,81 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>14.34</v>
+        <v>-97820</v>
       </c>
       <c r="D20" t="n">
-        <v>6.81</v>
+        <v>28.92</v>
       </c>
       <c r="E20" t="n">
-        <v>1.4</v>
+        <v>26.16</v>
       </c>
       <c r="F20" t="n">
-        <v>0.07000000000000001</v>
+        <v>8.52</v>
       </c>
       <c r="G20" t="n">
-        <v>35669</v>
+        <v>0.58</v>
       </c>
       <c r="H20" t="n">
-        <v>21.95</v>
+        <v>0.09</v>
       </c>
       <c r="I20" t="n">
-        <v>23.87</v>
+        <v>-101229</v>
       </c>
       <c r="J20" t="n">
-        <v>15.42</v>
+        <v>11.08</v>
       </c>
       <c r="K20" t="n">
-        <v>49.05</v>
+        <v>15.92</v>
       </c>
       <c r="L20" t="n">
-        <v>7.67</v>
+        <v>14.87</v>
       </c>
       <c r="M20" t="n">
-        <v>808359.03</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="N20" t="n">
-        <v>49.42</v>
+        <v>2011885.81</v>
       </c>
       <c r="O20" t="n">
-        <v>4.4</v>
+        <v>35.6</v>
       </c>
       <c r="P20" t="n">
-        <v>4.33</v>
+        <v>6.59</v>
       </c>
       <c r="Q20" t="n">
-        <v>283649</v>
+        <v>0.42</v>
       </c>
       <c r="R20" t="n">
-        <v>65446</v>
+        <v>91508</v>
       </c>
       <c r="S20" t="n">
-        <v>-44685</v>
-      </c>
-      <c r="T20" t="inlineStr">
+        <v>26461</v>
+      </c>
+      <c r="T20" t="n">
+        <v>37</v>
+      </c>
+      <c r="U20" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="U20" t="n">
+      <c r="V20" t="n">
         <v>23</v>
       </c>
-      <c r="V20" t="n">
-        <v>30.18695614094877</v>
+      <c r="W20" t="n">
+        <v>38.00805772489838</v>
+      </c>
+      <c r="X20" t="n">
+        <v>12.09139730993719</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>8.493112204756725</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>BANKBARODA</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1950,72 +2136,81 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>20.4</v>
+        <v>-6274</v>
       </c>
       <c r="D21" t="n">
-        <v>6.42</v>
+        <v>15.94</v>
       </c>
       <c r="E21" t="n">
-        <v>1.6</v>
+        <v>15.76</v>
       </c>
       <c r="F21" t="n">
-        <v>0.09</v>
+        <v>12.14</v>
       </c>
       <c r="G21" t="n">
-        <v>-59554</v>
+        <v>1.9</v>
       </c>
       <c r="H21" t="n">
-        <v>13.34</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I21" t="n">
-        <v>19.76</v>
+        <v>-7559</v>
       </c>
       <c r="J21" t="n">
-        <v>19.67</v>
+        <v>17.48</v>
       </c>
       <c r="K21" t="n">
-        <v>48.87</v>
+        <v>74.51000000000001</v>
       </c>
       <c r="L21" t="n">
-        <v>10</v>
+        <v>55.18</v>
       </c>
       <c r="M21" t="n">
-        <v>291917.42</v>
+        <v>6.33</v>
       </c>
       <c r="N21" t="n">
-        <v>31.49</v>
+        <v>590971.02</v>
       </c>
       <c r="O21" t="n">
-        <v>4.59</v>
+        <v>16.89</v>
       </c>
       <c r="P21" t="n">
-        <v>2.18</v>
+        <v>4.15</v>
       </c>
       <c r="Q21" t="n">
-        <v>47517</v>
+        <v>2.62</v>
       </c>
       <c r="R21" t="n">
-        <v>14145</v>
+        <v>118379</v>
       </c>
       <c r="S21" t="n">
-        <v>101</v>
-      </c>
-      <c r="T21" t="inlineStr">
+        <v>18869</v>
+      </c>
+      <c r="T21" t="n">
+        <v>4102</v>
+      </c>
+      <c r="U21" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="U21" t="n">
-        <v>30</v>
-      </c>
       <c r="V21" t="n">
-        <v>10.14749732259019</v>
+        <v>21</v>
+      </c>
+      <c r="W21" t="n">
+        <v>37.60943761161097</v>
+      </c>
+      <c r="X21" t="n">
+        <v>10.97340757490808</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>16.78883948962531</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CHOLAFIN</t>
+          <t>INDUSINDBK</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2024,66 +2219,75 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>17.46</v>
+        <v>-16843</v>
       </c>
       <c r="D22" t="n">
-        <v>6.86</v>
+        <v>19.56</v>
       </c>
       <c r="E22" t="n">
-        <v>21.21</v>
+        <v>14.25</v>
       </c>
       <c r="F22" t="n">
-        <v>0.12</v>
+        <v>6.89</v>
       </c>
       <c r="G22" t="n">
-        <v>-38538</v>
+        <v>1.88</v>
       </c>
       <c r="H22" t="n">
-        <v>21.94</v>
+        <v>0.09</v>
       </c>
       <c r="I22" t="n">
-        <v>23.36</v>
+        <v>-17468</v>
       </c>
       <c r="J22" t="n">
-        <v>22.28</v>
+        <v>15.5</v>
       </c>
       <c r="K22" t="n">
-        <v>48.86</v>
+        <v>22.08</v>
       </c>
       <c r="L22" t="n">
-        <v>10.4</v>
+        <v>15.9</v>
       </c>
       <c r="M22" t="n">
-        <v>971931.96</v>
+        <v>7.93</v>
       </c>
       <c r="N22" t="n">
-        <v>16.79</v>
+        <v>1807433.12</v>
       </c>
       <c r="O22" t="n">
-        <v>10.36</v>
+        <v>8.99</v>
       </c>
       <c r="P22" t="n">
-        <v>2.83</v>
+        <v>3.7</v>
       </c>
       <c r="Q22" t="n">
-        <v>19163</v>
+        <v>1.42</v>
       </c>
       <c r="R22" t="n">
-        <v>3420</v>
+        <v>45748</v>
       </c>
       <c r="S22" t="n">
-        <v>4548</v>
-      </c>
-      <c r="T22" t="inlineStr">
+        <v>8950</v>
+      </c>
+      <c r="T22" t="n">
+        <v>2978</v>
+      </c>
+      <c r="U22" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="U22" t="n">
-        <v>5</v>
-      </c>
       <c r="V22" t="n">
-        <v>25.98553091668698</v>
+        <v>14</v>
+      </c>
+      <c r="W22" t="n">
+        <v>33.69686056943905</v>
+      </c>
+      <c r="X22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>16.41029009859514</v>
       </c>
     </row>
   </sheetData>

</xml_diff>